<commit_message>
Implemented persistent data using Gson
</commit_message>
<xml_diff>
--- a/CMPS 3390 Project 2 Log.xlsx
+++ b/CMPS 3390 Project 2 Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swimm\Documents\[EDUCATION]\[SPRING 2026]\CMPS 3390 - Application Development (Royer)\Project 2\CMPS3390-Project-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5B0EA20-70B3-432C-A6EC-5E98342BEEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA386B88-EEA5-4CB0-A153-7463E15960D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>RESOURCE</t>
   </si>
@@ -117,9 +117,6 @@
     <t>https://www.tutorialspoint.com/gson/index.htm</t>
   </si>
   <si>
-    <t>How to use JSON in our project</t>
-  </si>
-  <si>
     <t>https://mvnrepository.com/artifact/com.google.code.gson/gson/2.13.2</t>
   </si>
   <si>
@@ -127,6 +124,15 @@
   </si>
   <si>
     <t>Install VS Code</t>
+  </si>
+  <si>
+    <t>https://howtodoinjava.com/gson/gson-typeadapter-for-inaccessibleobjectexception/</t>
+  </si>
+  <si>
+    <t>Handling Date and Time with Gson</t>
+  </si>
+  <si>
+    <t>How to use JSON in our project using Gson</t>
   </si>
 </sst>
 </file>
@@ -979,16 +985,22 @@
         <v>25</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D12" s="11">
         <v>2.0833333333333332E-2</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="12"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="11"/>
+      <c r="B13" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="11">
+        <v>6.9444444444444441E-3</v>
+      </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="12"/>
@@ -1060,16 +1072,16 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" s="5">
         <v>1</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">

</xml_diff>